<commit_message>
fix: référence directe au ValueSet IPS procedures-uv-ips pour l'additional binding SNOMED CT
Supprime la copie locale fr-core-vs-procedure-code-snomed (qui recopiait
le périmètre ECL de procedures-uv-ips) au profit d'une référence directe
au canonical http://hl7.org/fhir/uv/ips/ValueSet/procedures-uv-ips,
identique à celui utilisé par le parent EU Core procedure-eu-core.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> dfea65fe8da9834c6d63cd30ba69d86dc59b8a6c
</commit_message>
<xml_diff>
--- a/nr-doc-core-procedure/ig/ValueSet-fr-core-vs-procedure-code.xlsx
+++ b/nr-doc-core-procedure/ig/ValueSet-fr-core-vs-procedure-code.xlsx
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-16T15:06:55+00:00</t>
+    <t>2026-09-16T15:10:32+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -93,7 +93,7 @@
 - CCAM : terminologie facturante pour la production d'actes.
 - CISIS jdv-absent-or-unknown-procedure-cisis pour actes chirurgicaux inconnus ou absents.
 Deux additional bindings extensibles, portés par FRCoreProcedureProfile.code, complètent ce binding par défaut :
-- fr-core-vs-procedure-code-snomed (SNOMED CT) pour la demande d'acte ou de report d'actes à des fins internationales (en cours de validation en Europe).
+- ValueSet IPS procedures-uv-ips (SNOMED CT, identique au parent EU Core) pour la demande d'acte ou de report d'actes à des fins internationales (en cours de validation en Europe).
 - fr-core-vs-procedure-code-autre (CISIS "Autre acte") si l'acte n'est pas trouvé dans CCAM ni SNOMED CT.
 Si aucun code approprié n'est disponible, l'acte peut être décrit en texte libre.</t>
   </si>

</xml_diff>